<commit_message>
chore: sincroniza planilhas de gestao e relatorios atualizados
</commit_message>
<xml_diff>
--- a/paper_traning_lay0x0/sinais_lay0x0_gestao_2026-08-14.xlsx
+++ b/paper_traning_lay0x0/sinais_lay0x0_gestao_2026-08-14.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21df80ec97692de0/Documentos/GitHub/ARKAD_PROD/paper_traning_lay0x0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_2B593D9757F96841DF982A11591600B44111EA77" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6886548E-14C7-4A04-9E09-7962AD4C149A}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_2B593D9757F96841DF982A11591600B44111EA77" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{031E3862-BD19-4409-BCA0-96EAFF68F7CD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sinais" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -272,6 +285,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -640,6 +657,10 @@
       <c r="K2">
         <v>1.56</v>
       </c>
+      <c r="L2" t="str">
+        <f>IF(O2=1,"GREEN", "RED")</f>
+        <v>GREEN</v>
+      </c>
       <c r="N2" t="s">
         <v>20</v>
       </c>
@@ -681,6 +702,10 @@
       <c r="K3">
         <v>1.47</v>
       </c>
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L11" si="0">IF(O3=1,"GREEN", "RED")</f>
+        <v>GREEN</v>
+      </c>
       <c r="N3" t="s">
         <v>20</v>
       </c>
@@ -722,6 +747,10 @@
       <c r="K4">
         <v>1.47</v>
       </c>
+      <c r="L4" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N4" t="s">
         <v>20</v>
       </c>
@@ -763,6 +792,10 @@
       <c r="K5">
         <v>1.39</v>
       </c>
+      <c r="L5" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N5" t="s">
         <v>20</v>
       </c>
@@ -804,6 +837,10 @@
       <c r="K6">
         <v>1.92</v>
       </c>
+      <c r="L6" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N6" t="s">
         <v>20</v>
       </c>
@@ -845,6 +882,10 @@
       <c r="K7">
         <v>1.56</v>
       </c>
+      <c r="L7" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N7" t="s">
         <v>20</v>
       </c>
@@ -886,6 +927,10 @@
       <c r="K8">
         <v>1.39</v>
       </c>
+      <c r="L8" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N8" t="s">
         <v>20</v>
       </c>
@@ -927,8 +972,15 @@
       <c r="K9">
         <v>1.85</v>
       </c>
+      <c r="L9" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N9" t="s">
         <v>20</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -965,8 +1017,15 @@
       <c r="K10">
         <v>2.5</v>
       </c>
+      <c r="L10" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N10" t="s">
         <v>20</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
@@ -1003,8 +1062,15 @@
       <c r="K11">
         <v>2</v>
       </c>
+      <c r="L11" t="str">
+        <f t="shared" si="0"/>
+        <v>GREEN</v>
+      </c>
       <c r="N11" t="s">
         <v>20</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>